<commit_message>
cleared __init__ from MainApp
</commit_message>
<xml_diff>
--- a/data/outputs/table_status_analysis.xlsx
+++ b/data/outputs/table_status_analysis.xlsx
@@ -17,7 +17,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Max People per Hour" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Table Performance'!$A$1:$L$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Table Performance'!$A$1:$L$9</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -622,7 +622,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -636,17 +636,17 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>2024-11-19 17:09:45</t>
+          <t>2024-11-19 21:30:59</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>00:00:02</t>
+          <t>00:00:24</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>Afternoon</t>
+          <t>Evening</t>
         </is>
       </c>
     </row>
@@ -661,17 +661,17 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2024-11-19 17:09:45</t>
+          <t>2024-11-19 21:30:59</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>00:00:02</t>
+          <t>00:00:24</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Afternoon</t>
+          <t>Evening</t>
         </is>
       </c>
     </row>
@@ -686,17 +686,17 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2024-11-19 17:09:45</t>
+          <t>2024-11-19 21:30:59</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>00:00:02</t>
+          <t>00:00:24</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Afternoon</t>
+          <t>Evening</t>
         </is>
       </c>
     </row>
@@ -711,17 +711,17 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2024-11-19 17:09:45</t>
+          <t>2024-11-19 21:30:59</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>00:00:02</t>
+          <t>00:00:24</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Afternoon</t>
+          <t>Evening</t>
         </is>
       </c>
     </row>
@@ -736,17 +736,17 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2024-11-19 17:09:45</t>
+          <t>2024-11-19 21:30:59</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>00:00:02</t>
+          <t>00:00:24</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Afternoon</t>
+          <t>Evening</t>
         </is>
       </c>
     </row>
@@ -761,17 +761,17 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2024-11-19 17:09:45</t>
+          <t>2024-11-19 21:30:59</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>00:00:02</t>
+          <t>00:00:24</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Afternoon</t>
+          <t>Evening</t>
         </is>
       </c>
     </row>
@@ -786,17 +786,17 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2024-11-19 17:09:45</t>
+          <t>2024-11-19 21:30:59</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>00:00:02</t>
+          <t>00:00:24</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Afternoon</t>
+          <t>Evening</t>
         </is>
       </c>
     </row>
@@ -811,67 +811,17 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2024-11-19 17:09:45</t>
+          <t>2024-11-19 21:30:59</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>00:00:02</t>
+          <t>00:00:24</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Afternoon</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="n">
-        <v>9</v>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>available</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>2024-11-19 17:09:45</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>00:00:02</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>Afternoon</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="n">
-        <v>10</v>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>available</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>2024-11-19 17:09:45</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>00:00:02</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>Afternoon</t>
+          <t>Evening</t>
         </is>
       </c>
     </row>
@@ -942,12 +892,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>00:00:02</t>
+          <t>00:00:24</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>00:00:02</t>
+          <t>00:00:24</t>
         </is>
       </c>
     </row>
@@ -977,7 +927,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L11"/>
+  <dimension ref="A1:L9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1048,7 +998,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>00:00:02</t>
+          <t>00:00:24</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -1073,7 +1023,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>00:00:02</t>
+          <t>00:00:24</t>
         </is>
       </c>
       <c r="H2" t="n">
@@ -1098,7 +1048,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>00:00:02</t>
+          <t>00:00:24</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1123,7 +1073,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>00:00:02</t>
+          <t>00:00:24</t>
         </is>
       </c>
       <c r="H3" t="n">
@@ -1148,7 +1098,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>00:00:02</t>
+          <t>00:00:24</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -1173,7 +1123,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>00:00:02</t>
+          <t>00:00:24</t>
         </is>
       </c>
       <c r="H4" t="n">
@@ -1198,7 +1148,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>00:00:02</t>
+          <t>00:00:24</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -1223,7 +1173,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>00:00:02</t>
+          <t>00:00:24</t>
         </is>
       </c>
       <c r="H5" t="n">
@@ -1248,7 +1198,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>00:00:02</t>
+          <t>00:00:24</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -1273,7 +1223,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>00:00:02</t>
+          <t>00:00:24</t>
         </is>
       </c>
       <c r="H6" t="n">
@@ -1298,7 +1248,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>00:00:02</t>
+          <t>00:00:24</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1323,7 +1273,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>00:00:02</t>
+          <t>00:00:24</t>
         </is>
       </c>
       <c r="H7" t="n">
@@ -1348,7 +1298,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>00:00:02</t>
+          <t>00:00:24</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1373,7 +1323,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>00:00:02</t>
+          <t>00:00:24</t>
         </is>
       </c>
       <c r="H8" t="n">
@@ -1398,7 +1348,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>00:00:02</t>
+          <t>00:00:24</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1423,7 +1373,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>00:00:02</t>
+          <t>00:00:24</t>
         </is>
       </c>
       <c r="H9" t="n">
@@ -1442,108 +1392,8 @@
         <v>-0.1</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="n">
-        <v>9</v>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>00:00:02</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>00:00:00</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>00:00:00</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>00:00:00</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>00:00:00</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>00:00:02</t>
-        </is>
-      </c>
-      <c r="H10" t="n">
-        <v>1</v>
-      </c>
-      <c r="I10" t="n">
-        <v>0</v>
-      </c>
-      <c r="J10" t="n">
-        <v>0</v>
-      </c>
-      <c r="K10" t="n">
-        <v>0</v>
-      </c>
-      <c r="L10" t="n">
-        <v>-0.1</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="n">
-        <v>10</v>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>00:00:02</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>00:00:00</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>00:00:00</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>00:00:00</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>00:00:00</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>00:00:02</t>
-        </is>
-      </c>
-      <c r="H11" t="n">
-        <v>1</v>
-      </c>
-      <c r="I11" t="n">
-        <v>0</v>
-      </c>
-      <c r="J11" t="n">
-        <v>0</v>
-      </c>
-      <c r="K11" t="n">
-        <v>0</v>
-      </c>
-      <c r="L11" t="n">
-        <v>-0.1</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:L11"/>
+  <autoFilter ref="A1:L9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1586,11 +1436,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>